<commit_message>
Adapted some figures and models and the insurance value calculation
I hope these were one of the last edits to my script. Of course I have to prepare them for publishing at one point. Also, I have to update some figures probably to make the suitable for publishing.
</commit_message>
<xml_diff>
--- a/Data Analysis/1_Data/economic_MF_final.xlsx
+++ b/Data Analysis/1_Data/economic_MF_final.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W79"/>
+  <dimension ref="A1:AB79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -447,27 +447,52 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
+          <t>SOC_costs_mid</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>SOC_costs_lo</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>SOC_costs_hi</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_mid</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_lo</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_hi</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_mid_adj</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_lo_adj</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>costs_total_hi_adj</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>meanSR</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>SOC_costs_mid</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>SOC_costs_lo</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>SOC_costs_hi</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>costs_total_mid</t>
         </is>
       </c>
     </row>
@@ -530,17 +555,35 @@
       <c r="R2">
         <v>-50.28157516499095</v>
       </c>
+      <c r="S2">
+        <v>776.0019362477558</v>
+      </c>
       <c r="T2">
-        <v>776.0019362477558</v>
+        <v>194.0004840619389</v>
       </c>
       <c r="U2">
-        <v>194.0004840619389</v>
+        <v>2069.338496660682</v>
       </c>
       <c r="V2">
-        <v>2069.338496660682</v>
+        <v>1199.796918580594</v>
       </c>
       <c r="W2">
-        <v>1199.796918580594</v>
+        <v>637.6985898975859</v>
+      </c>
+      <c r="X2">
+        <v>2473.230355490711</v>
+      </c>
+      <c r="Y2">
+        <v>1174.819290662734</v>
+      </c>
+      <c r="Z2">
+        <v>612.7209619797263</v>
+      </c>
+      <c r="AA2">
+        <v>2448.252727572852</v>
+      </c>
+      <c r="AB2">
+        <v>11.83333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -602,17 +645,35 @@
       <c r="R3">
         <v>-62.7502337238665</v>
       </c>
+      <c r="S3">
+        <v>7.583391783192281</v>
+      </c>
       <c r="T3">
-        <v>7.583391783192281</v>
+        <v>1.89584794579807</v>
       </c>
       <c r="U3">
-        <v>1.89584794579807</v>
+        <v>20.22237808851275</v>
       </c>
       <c r="V3">
-        <v>20.22237808851275</v>
+        <v>332.0857615465974</v>
       </c>
       <c r="W3">
-        <v>332.0857615465974</v>
+        <v>351.236851891567</v>
+      </c>
+      <c r="X3">
+        <v>319.8861136695541</v>
+      </c>
+      <c r="Y3">
+        <v>309.9722182278929</v>
+      </c>
+      <c r="Z3">
+        <v>329.1233085728625</v>
+      </c>
+      <c r="AA3">
+        <v>297.7725703508496</v>
+      </c>
+      <c r="AB3">
+        <v>5.728813559322034</v>
       </c>
     </row>
     <row r="4">
@@ -674,17 +735,35 @@
       <c r="R4">
         <v>-188.9905626286803</v>
       </c>
+      <c r="S4">
+        <v>74.56707340401853</v>
+      </c>
       <c r="T4">
-        <v>74.56707340401853</v>
+        <v>18.64176835100463</v>
       </c>
       <c r="U4">
-        <v>18.64176835100463</v>
+        <v>198.8455290773827</v>
       </c>
       <c r="V4">
-        <v>198.8455290773827</v>
+        <v>269.0197711049724</v>
       </c>
       <c r="W4">
-        <v>269.0197711049724</v>
+        <v>287.9032304258111</v>
+      </c>
+      <c r="X4">
+        <v>318.4894624044839</v>
+      </c>
+      <c r="Y4">
+        <v>228.2054794829228</v>
+      </c>
+      <c r="Z4">
+        <v>247.0889388037616</v>
+      </c>
+      <c r="AA4">
+        <v>277.6751707824344</v>
+      </c>
+      <c r="AB4">
+        <v>6.186440677966102</v>
       </c>
     </row>
     <row r="5">
@@ -746,17 +825,35 @@
       <c r="R5">
         <v>-162.3022324266065</v>
       </c>
+      <c r="S5">
+        <v>-381.4278283481973</v>
+      </c>
       <c r="T5">
-        <v>-381.4278283481973</v>
+        <v>-95.35695708704932</v>
       </c>
       <c r="U5">
-        <v>-95.35695708704932</v>
+        <v>-1017.140875595193</v>
       </c>
       <c r="V5">
-        <v>-1017.140875595193</v>
+        <v>-44.23153113298775</v>
       </c>
       <c r="W5">
-        <v>-44.23153113298775</v>
+        <v>306.0839737970252</v>
+      </c>
+      <c r="X5">
+        <v>-744.1892120488487</v>
+      </c>
+      <c r="Y5">
+        <v>-97.50655458481287</v>
+      </c>
+      <c r="Z5">
+        <v>252.8089503452001</v>
+      </c>
+      <c r="AA5">
+        <v>-797.4642355006738</v>
+      </c>
+      <c r="AB5">
+        <v>3.35</v>
       </c>
     </row>
     <row r="6">
@@ -818,17 +915,35 @@
       <c r="R6">
         <v>-130.8609161569784</v>
       </c>
+      <c r="S6">
+        <v>-405.2626142571454</v>
+      </c>
       <c r="T6">
-        <v>-405.2626142571454</v>
+        <v>-101.3156535642864</v>
       </c>
       <c r="U6">
-        <v>-101.3156535642864</v>
+        <v>-1080.700304685721</v>
       </c>
       <c r="V6">
-        <v>-1080.700304685721</v>
+        <v>-90.0137311573996</v>
       </c>
       <c r="W6">
-        <v>-90.0137311573996</v>
+        <v>265.73234218093</v>
+      </c>
+      <c r="X6">
+        <v>-817.250534231446</v>
+      </c>
+      <c r="Y6">
+        <v>-186.8008859237345</v>
+      </c>
+      <c r="Z6">
+        <v>168.945187414595</v>
+      </c>
+      <c r="AA6">
+        <v>-914.0376889977808</v>
+      </c>
+      <c r="AB6">
+        <v>1.864406779661017</v>
       </c>
     </row>
     <row r="7">
@@ -890,17 +1005,35 @@
       <c r="R7">
         <v>-30.39190942733287</v>
       </c>
+      <c r="S7">
+        <v>212.5784837509758</v>
+      </c>
       <c r="T7">
-        <v>212.5784837509758</v>
+        <v>53.14462093774394</v>
       </c>
       <c r="U7">
-        <v>53.14462093774394</v>
+        <v>566.8759566692687</v>
       </c>
       <c r="V7">
-        <v>566.8759566692687</v>
+        <v>519.165044223625</v>
       </c>
       <c r="W7">
-        <v>519.165044223625</v>
+        <v>371.7613122253791</v>
+      </c>
+      <c r="X7">
+        <v>861.432386326932</v>
+      </c>
+      <c r="Y7">
+        <v>493.5979868701391</v>
+      </c>
+      <c r="Z7">
+        <v>346.1942548718931</v>
+      </c>
+      <c r="AA7">
+        <v>835.8653289734461</v>
+      </c>
+      <c r="AB7">
+        <v>12.89830508474576</v>
       </c>
     </row>
     <row r="8">
@@ -962,17 +1095,35 @@
       <c r="R8">
         <v>-140.0203770131957</v>
       </c>
+      <c r="S8">
+        <v>-373.4422893248743</v>
+      </c>
       <c r="T8">
-        <v>-373.4422893248743</v>
+        <v>-93.36057233121856</v>
       </c>
       <c r="U8">
-        <v>-93.36057233121856</v>
+        <v>-995.8461048663313</v>
       </c>
       <c r="V8">
-        <v>-995.8461048663313</v>
+        <v>-268.3569332170637</v>
       </c>
       <c r="W8">
-        <v>-268.3569332170637</v>
+        <v>67.14951634431534</v>
+      </c>
+      <c r="X8">
+        <v>-946.1854813262441</v>
+      </c>
+      <c r="Y8">
+        <v>-299.5629172595596</v>
+      </c>
+      <c r="Z8">
+        <v>35.94353230181943</v>
+      </c>
+      <c r="AA8">
+        <v>-977.39146536874</v>
+      </c>
+      <c r="AB8">
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -1034,17 +1185,35 @@
       <c r="R9">
         <v>-229.3370740969741</v>
       </c>
+      <c r="S9">
+        <v>-356.7084314993093</v>
+      </c>
       <c r="T9">
-        <v>-356.7084314993093</v>
+        <v>-89.17710787482731</v>
       </c>
       <c r="U9">
-        <v>-89.17710787482731</v>
+        <v>-951.2224839981581</v>
       </c>
       <c r="V9">
-        <v>-951.2224839981581</v>
+        <v>-112.489464672712</v>
       </c>
       <c r="W9">
-        <v>-112.489464672712</v>
+        <v>245.8211174484889</v>
+      </c>
+      <c r="X9">
+        <v>-797.7827756682797</v>
+      </c>
+      <c r="Y9">
+        <v>-164.1507470642426</v>
+      </c>
+      <c r="Z9">
+        <v>194.1598350569583</v>
+      </c>
+      <c r="AA9">
+        <v>-849.4440580598102</v>
+      </c>
+      <c r="AB9">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1106,17 +1275,35 @@
       <c r="R10">
         <v>-106.6752976432115</v>
       </c>
+      <c r="S10">
+        <v>-453.0081391389492</v>
+      </c>
       <c r="T10">
-        <v>-453.0081391389492</v>
+        <v>-113.2520347847373</v>
       </c>
       <c r="U10">
-        <v>-113.2520347847373</v>
+        <v>-1208.021704370531</v>
       </c>
       <c r="V10">
-        <v>-1208.021704370531</v>
+        <v>-440.8477004595866</v>
       </c>
       <c r="W10">
-        <v>-440.8477004595866</v>
+        <v>-58.8659574549369</v>
+      </c>
+      <c r="X10">
+        <v>-1238.086904341606</v>
+      </c>
+      <c r="Y10">
+        <v>-461.0820232260895</v>
+      </c>
+      <c r="Z10">
+        <v>-79.10028022143968</v>
+      </c>
+      <c r="AA10">
+        <v>-1258.321227108109</v>
+      </c>
+      <c r="AB10">
+        <v>0.9523809523809523</v>
       </c>
     </row>
     <row r="11">
@@ -1178,17 +1365,35 @@
       <c r="R11">
         <v>-55.81306805400369</v>
       </c>
+      <c r="S11">
+        <v>1022.72996477033</v>
+      </c>
       <c r="T11">
-        <v>1022.72996477033</v>
+        <v>255.6824911925825</v>
       </c>
       <c r="U11">
-        <v>255.6824911925825</v>
+        <v>2727.279906054213</v>
       </c>
       <c r="V11">
-        <v>2727.279906054213</v>
+        <v>1340.228588122322</v>
       </c>
       <c r="W11">
-        <v>1340.228588122322</v>
+        <v>595.2737873159515</v>
+      </c>
+      <c r="X11">
+        <v>3022.685856634829</v>
+      </c>
+      <c r="Y11">
+        <v>1315.037476283804</v>
+      </c>
+      <c r="Z11">
+        <v>570.0826754774328</v>
+      </c>
+      <c r="AA11">
+        <v>2997.49474479631</v>
+      </c>
+      <c r="AB11">
+        <v>11.03333333333333</v>
       </c>
     </row>
     <row r="12">
@@ -1250,17 +1455,35 @@
       <c r="R12">
         <v>-162.4702296753888</v>
       </c>
+      <c r="S12">
+        <v>-370.1816630423123</v>
+      </c>
       <c r="T12">
-        <v>-370.1816630423123</v>
+        <v>-92.54541576057808</v>
       </c>
       <c r="U12">
-        <v>-92.54541576057808</v>
+        <v>-987.1511014461662</v>
       </c>
       <c r="V12">
-        <v>-987.1511014461662</v>
+        <v>25.22115899744279</v>
       </c>
       <c r="W12">
-        <v>25.22115899744279</v>
+        <v>367.1685388590184</v>
+      </c>
+      <c r="X12">
+        <v>-656.0594119862524</v>
+      </c>
+      <c r="Y12">
+        <v>-22.7144506118965</v>
+      </c>
+      <c r="Z12">
+        <v>319.2329292496792</v>
+      </c>
+      <c r="AA12">
+        <v>-703.9950215955917</v>
+      </c>
+      <c r="AB12">
+        <v>5.3</v>
       </c>
     </row>
     <row r="13">
@@ -1322,17 +1545,35 @@
       <c r="R13">
         <v>-148.852252336754</v>
       </c>
+      <c r="S13">
+        <v>-168.5018317652187</v>
+      </c>
       <c r="T13">
-        <v>-168.5018317652187</v>
+        <v>-42.12545794130468</v>
       </c>
       <c r="U13">
-        <v>-42.12545794130468</v>
+        <v>-449.3382180405833</v>
       </c>
       <c r="V13">
-        <v>-449.3382180405833</v>
+        <v>215.7509264607076</v>
       </c>
       <c r="W13">
-        <v>215.7509264607076</v>
+        <v>401.0479835012534</v>
+      </c>
+      <c r="X13">
+        <v>-124.0061430312888</v>
+      </c>
+      <c r="Y13">
+        <v>154.4443195002807</v>
+      </c>
+      <c r="Z13">
+        <v>339.7413765408265</v>
+      </c>
+      <c r="AA13">
+        <v>-185.3127499917157</v>
+      </c>
+      <c r="AB13">
+        <v>3.2</v>
       </c>
     </row>
     <row r="14">
@@ -1394,17 +1635,35 @@
       <c r="R14">
         <v>-40.78101627379836</v>
       </c>
+      <c r="S14">
+        <v>433.4735654111012</v>
+      </c>
       <c r="T14">
-        <v>433.4735654111012</v>
+        <v>108.3683913527753</v>
       </c>
       <c r="U14">
-        <v>108.3683913527753</v>
+        <v>1155.929507762937</v>
       </c>
       <c r="V14">
-        <v>1155.929507762937</v>
+        <v>665.7460203906239</v>
       </c>
       <c r="W14">
-        <v>665.7460203906239</v>
+        <v>356.7833319406766</v>
+      </c>
+      <c r="X14">
+        <v>1372.059477134081</v>
+      </c>
+      <c r="Y14">
+        <v>642.0721786034248</v>
+      </c>
+      <c r="Z14">
+        <v>333.1094901534775</v>
+      </c>
+      <c r="AA14">
+        <v>1348.385635346882</v>
+      </c>
+      <c r="AB14">
+        <v>6.559322033898305</v>
       </c>
     </row>
     <row r="15">
@@ -1466,17 +1725,35 @@
       <c r="R15">
         <v>-92.49525164652148</v>
       </c>
+      <c r="S15">
+        <v>-607.3755880406841</v>
+      </c>
       <c r="T15">
-        <v>-607.3755880406841</v>
+        <v>-151.843897010171</v>
       </c>
       <c r="U15">
-        <v>-151.843897010171</v>
+        <v>-1619.668234775158</v>
       </c>
       <c r="V15">
-        <v>-1619.668234775158</v>
+        <v>-567.2566809043824</v>
       </c>
       <c r="W15">
-        <v>-567.2566809043824</v>
+        <v>-75.1122860971212</v>
+      </c>
+      <c r="X15">
+        <v>-1616.162031415604</v>
+      </c>
+      <c r="Y15">
+        <v>-613.1997392876918</v>
+      </c>
+      <c r="Z15">
+        <v>-121.0553444804307</v>
+      </c>
+      <c r="AA15">
+        <v>-1662.105089798914</v>
+      </c>
+      <c r="AB15">
+        <v>0.95</v>
       </c>
     </row>
     <row r="16">
@@ -1538,17 +1815,35 @@
       <c r="R16">
         <v>-27.27674853955119</v>
       </c>
+      <c r="S16">
+        <v>-637.9332337409667</v>
+      </c>
       <c r="T16">
-        <v>-637.9332337409667</v>
+        <v>-159.4833084352417</v>
       </c>
       <c r="U16">
-        <v>-159.4833084352417</v>
+        <v>-1701.155289975911</v>
       </c>
       <c r="V16">
-        <v>-1701.155289975911</v>
+        <v>-478.7079655648573</v>
       </c>
       <c r="W16">
-        <v>-478.7079655648573</v>
+        <v>10.53900603777336</v>
+      </c>
+      <c r="X16">
+        <v>-1552.727068096707</v>
+      </c>
+      <c r="Y16">
+        <v>-505.2378736507658</v>
+      </c>
+      <c r="Z16">
+        <v>-15.99090204813513</v>
+      </c>
+      <c r="AA16">
+        <v>-1579.256976182616</v>
+      </c>
+      <c r="AB16">
+        <v>1.983050847457627</v>
       </c>
     </row>
     <row r="17">
@@ -1610,17 +1905,35 @@
       <c r="R17">
         <v>-69.41329029307803</v>
       </c>
+      <c r="S17">
+        <v>-998.2419574417249</v>
+      </c>
       <c r="T17">
-        <v>-998.2419574417249</v>
+        <v>-249.5604893604312</v>
       </c>
       <c r="U17">
-        <v>-249.5604893604312</v>
+        <v>-2661.978553177933</v>
       </c>
       <c r="V17">
-        <v>-2661.978553177933</v>
+        <v>-835.1601508826228</v>
       </c>
       <c r="W17">
-        <v>-835.1601508826228</v>
+        <v>-59.00258872698569</v>
+      </c>
+      <c r="X17">
+        <v>-2526.372840693175</v>
+      </c>
+      <c r="Y17">
+        <v>-862.2051580861246</v>
+      </c>
+      <c r="Z17">
+        <v>-86.04759593048749</v>
+      </c>
+      <c r="AA17">
+        <v>-2553.417847896676</v>
+      </c>
+      <c r="AB17">
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -1682,17 +1995,35 @@
       <c r="R18">
         <v>-52.17060611591119</v>
       </c>
+      <c r="S18">
+        <v>-757.7101452362072</v>
+      </c>
       <c r="T18">
-        <v>-757.7101452362072</v>
+        <v>-189.4275363090518</v>
       </c>
       <c r="U18">
-        <v>-189.4275363090518</v>
+        <v>-2020.560387296552</v>
       </c>
       <c r="V18">
-        <v>-2020.560387296552</v>
+        <v>-720.5702479627346</v>
       </c>
       <c r="W18">
-        <v>-720.5702479627346</v>
+        <v>-131.6367741146976</v>
+      </c>
+      <c r="X18">
+        <v>-2004.071354943961</v>
+      </c>
+      <c r="Y18">
+        <v>-735.2204064114636</v>
+      </c>
+      <c r="Z18">
+        <v>-146.2869325634267</v>
+      </c>
+      <c r="AA18">
+        <v>-2018.72151339269</v>
+      </c>
+      <c r="AB18">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -1754,17 +2085,35 @@
       <c r="R19">
         <v>-52.46373763961006</v>
       </c>
+      <c r="S19">
+        <v>-744.369023474728</v>
+      </c>
       <c r="T19">
-        <v>-744.369023474728</v>
+        <v>-186.092255868682</v>
       </c>
       <c r="U19">
-        <v>-186.092255868682</v>
+        <v>-1984.984062599275</v>
       </c>
       <c r="V19">
-        <v>-1984.984062599275</v>
+        <v>-500.4924387744687</v>
       </c>
       <c r="W19">
-        <v>-500.4924387744687</v>
+        <v>78.55122498058967</v>
+      </c>
+      <c r="X19">
+        <v>-1761.874374048028</v>
+      </c>
+      <c r="Y19">
+        <v>-533.2304330549545</v>
+      </c>
+      <c r="Z19">
+        <v>45.81323070010387</v>
+      </c>
+      <c r="AA19">
+        <v>-1794.612368328514</v>
+      </c>
+      <c r="AB19">
+        <v>3.559322033898305</v>
       </c>
     </row>
     <row r="20">
@@ -1826,17 +2175,35 @@
       <c r="R20">
         <v>-80.56385715887156</v>
       </c>
+      <c r="S20">
+        <v>-156.5795148059204</v>
+      </c>
       <c r="T20">
-        <v>-156.5795148059204</v>
+        <v>-39.14487870148009</v>
       </c>
       <c r="U20">
-        <v>-39.14487870148009</v>
+        <v>-417.5453728157876</v>
       </c>
       <c r="V20">
-        <v>-417.5453728157876</v>
+        <v>419.1702552231611</v>
       </c>
       <c r="W20">
-        <v>419.1702552231611</v>
+        <v>568.4947514529881</v>
+      </c>
+      <c r="X20">
+        <v>126.3145370879073</v>
+      </c>
+      <c r="Y20">
+        <v>395.6144780887071</v>
+      </c>
+      <c r="Z20">
+        <v>544.9389743185341</v>
+      </c>
+      <c r="AA20">
+        <v>102.7587599534533</v>
+      </c>
+      <c r="AB20">
+        <v>12.15254237288136</v>
       </c>
     </row>
     <row r="21">
@@ -1898,17 +2265,35 @@
       <c r="R21">
         <v>-23.97763894200598</v>
       </c>
+      <c r="S21">
+        <v>72.5154982273032</v>
+      </c>
       <c r="T21">
-        <v>72.5154982273032</v>
+        <v>18.1288745568258</v>
       </c>
       <c r="U21">
-        <v>18.1288745568258</v>
+        <v>193.3746619394752</v>
       </c>
       <c r="V21">
-        <v>193.3746619394752</v>
+        <v>221.6466975868286</v>
       </c>
       <c r="W21">
-        <v>221.6466975868286</v>
+        <v>176.7512226642285</v>
+      </c>
+      <c r="X21">
+        <v>333.0147125511232</v>
+      </c>
+      <c r="Y21">
+        <v>182.0443655397778</v>
+      </c>
+      <c r="Z21">
+        <v>137.1488906171778</v>
+      </c>
+      <c r="AA21">
+        <v>293.4123805040724</v>
+      </c>
+      <c r="AB21">
+        <v>3.694915254237288</v>
       </c>
     </row>
     <row r="22">
@@ -1970,17 +2355,35 @@
       <c r="R22">
         <v>-45.07948438017191</v>
       </c>
+      <c r="S22">
+        <v>822.0031998972684</v>
+      </c>
       <c r="T22">
-        <v>822.0031998972684</v>
+        <v>205.5007999743171</v>
       </c>
       <c r="U22">
-        <v>205.5007999743171</v>
+        <v>2192.008533059382</v>
       </c>
       <c r="V22">
-        <v>2192.008533059382</v>
+        <v>1285.335184067434</v>
       </c>
       <c r="W22">
-        <v>1285.335184067434</v>
+        <v>686.6767467116343</v>
+      </c>
+      <c r="X22">
+        <v>2637.496554662397</v>
+      </c>
+      <c r="Y22">
+        <v>1262.956351865978</v>
+      </c>
+      <c r="Z22">
+        <v>664.297914510178</v>
+      </c>
+      <c r="AA22">
+        <v>2615.11772246094</v>
+      </c>
+      <c r="AB22">
+        <v>3.6</v>
       </c>
     </row>
     <row r="23">
@@ -2042,17 +2445,35 @@
       <c r="R23">
         <v>-17.7815422654048</v>
       </c>
+      <c r="S23">
+        <v>-50.02277013860132</v>
+      </c>
       <c r="T23">
-        <v>-50.02277013860132</v>
+        <v>-12.50569253465033</v>
       </c>
       <c r="U23">
-        <v>-12.50569253465033</v>
+        <v>-133.3940537029368</v>
       </c>
       <c r="V23">
-        <v>-133.3940537029368</v>
+        <v>143.8596715655736</v>
       </c>
       <c r="W23">
-        <v>143.8596715655736</v>
+        <v>188.4152763162473</v>
+      </c>
+      <c r="X23">
+        <v>53.44986085451541</v>
+      </c>
+      <c r="Y23">
+        <v>113.3344522565354</v>
+      </c>
+      <c r="Z23">
+        <v>157.8900570072091</v>
+      </c>
+      <c r="AA23">
+        <v>22.92464154547721</v>
+      </c>
+      <c r="AB23">
+        <v>1.983050847457627</v>
       </c>
     </row>
     <row r="24">
@@ -2114,17 +2535,35 @@
       <c r="R24">
         <v>-120.8238153226634</v>
       </c>
+      <c r="S24">
+        <v>-216.7298338907898</v>
+      </c>
       <c r="T24">
-        <v>-216.7298338907898</v>
+        <v>-54.18245847269746</v>
       </c>
       <c r="U24">
-        <v>-54.18245847269746</v>
+        <v>-577.9462237087729</v>
       </c>
       <c r="V24">
-        <v>-577.9462237087729</v>
+        <v>-137.527507048459</v>
       </c>
       <c r="W24">
-        <v>-137.527507048459</v>
+        <v>72.84596193485439</v>
+      </c>
+      <c r="X24">
+        <v>-546.569990431663</v>
+      </c>
+      <c r="Y24">
+        <v>-167.0975023124461</v>
+      </c>
+      <c r="Z24">
+        <v>43.27596667086719</v>
+      </c>
+      <c r="AA24">
+        <v>-576.1399856956501</v>
+      </c>
+      <c r="AB24">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -2186,17 +2625,35 @@
       <c r="R25">
         <v>-45.6945025391969</v>
       </c>
+      <c r="S25">
+        <v>-70.16476144728868</v>
+      </c>
       <c r="T25">
-        <v>-70.16476144728868</v>
+        <v>-17.54119036182217</v>
       </c>
       <c r="U25">
-        <v>-17.54119036182217</v>
+        <v>-187.1060305261032</v>
       </c>
       <c r="V25">
-        <v>-187.1060305261032</v>
+        <v>71.88984265032799</v>
       </c>
       <c r="W25">
-        <v>71.88984265032799</v>
+        <v>142.6008209908933</v>
+      </c>
+      <c r="X25">
+        <v>-63.13883368358529</v>
+      </c>
+      <c r="Y25">
+        <v>15.51834537401299</v>
+      </c>
+      <c r="Z25">
+        <v>86.22932371457827</v>
+      </c>
+      <c r="AA25">
+        <v>-119.5103309599003</v>
+      </c>
+      <c r="AB25">
+        <v>0.9833333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -2258,17 +2715,35 @@
       <c r="R26">
         <v>-59.87185375948937</v>
       </c>
+      <c r="S26">
+        <v>458.1313522679775</v>
+      </c>
       <c r="T26">
-        <v>458.1313522679775</v>
+        <v>114.5328380669944</v>
       </c>
       <c r="U26">
-        <v>114.5328380669944</v>
+        <v>1221.68360604794</v>
       </c>
       <c r="V26">
-        <v>1221.68360604794</v>
+        <v>741.9088060560481</v>
       </c>
       <c r="W26">
-        <v>741.9088060560481</v>
+        <v>422.0095673015295</v>
+      </c>
+      <c r="X26">
+        <v>1481.761784389546</v>
+      </c>
+      <c r="Y26">
+        <v>726.1001737160364</v>
+      </c>
+      <c r="Z26">
+        <v>406.2009349615178</v>
+      </c>
+      <c r="AA26">
+        <v>1465.953152049534</v>
+      </c>
+      <c r="AB26">
+        <v>3.677966101694915</v>
       </c>
     </row>
     <row r="27">
@@ -2330,17 +2805,35 @@
       <c r="R27">
         <v>-48.31947164076955</v>
       </c>
+      <c r="S27">
+        <v>-417.5614356405866</v>
+      </c>
       <c r="T27">
-        <v>-417.5614356405866</v>
+        <v>-104.3903589101467</v>
       </c>
       <c r="U27">
-        <v>-104.3903589101467</v>
+        <v>-1113.497161708231</v>
       </c>
       <c r="V27">
-        <v>-1113.497161708231</v>
+        <v>-293.6516502873247</v>
       </c>
       <c r="W27">
-        <v>-293.6516502873247</v>
+        <v>38.64588396758651</v>
+      </c>
+      <c r="X27">
+        <v>-1008.71383387944</v>
+      </c>
+      <c r="Y27">
+        <v>-320.4291188051111</v>
+      </c>
+      <c r="Z27">
+        <v>11.8684154498001</v>
+      </c>
+      <c r="AA27">
+        <v>-1035.491302397227</v>
+      </c>
+      <c r="AB27">
+        <v>1.627118644067797</v>
       </c>
     </row>
     <row r="28">
@@ -2402,17 +2895,35 @@
       <c r="R28">
         <v>-23.98385578133442</v>
       </c>
+      <c r="S28">
+        <v>-152.817217983223</v>
+      </c>
       <c r="T28">
-        <v>-152.817217983223</v>
+        <v>-38.20430449580575</v>
       </c>
       <c r="U28">
-        <v>-38.20430449580575</v>
+        <v>-407.5125812885947</v>
       </c>
       <c r="V28">
-        <v>-407.5125812885947</v>
+        <v>40.03281807292754</v>
       </c>
       <c r="W28">
-        <v>40.03281807292754</v>
+        <v>164.1393411404563</v>
+      </c>
+      <c r="X28">
+        <v>-224.1561548125557</v>
+      </c>
+      <c r="Y28">
+        <v>13.32896056403143</v>
+      </c>
+      <c r="Z28">
+        <v>137.4354836315602</v>
+      </c>
+      <c r="AA28">
+        <v>-250.8600123214518</v>
+      </c>
+      <c r="AB28">
+        <v>3.933333333333333</v>
       </c>
     </row>
     <row r="29">
@@ -2474,17 +2985,35 @@
       <c r="R29">
         <v>-26.07845498112912</v>
       </c>
+      <c r="S29">
+        <v>446.5867656201178</v>
+      </c>
       <c r="T29">
-        <v>446.5867656201178</v>
+        <v>111.6466914050294</v>
       </c>
       <c r="U29">
-        <v>111.6466914050294</v>
+        <v>1190.898041653647</v>
       </c>
       <c r="V29">
-        <v>1190.898041653647</v>
+        <v>824.3725758992462</v>
       </c>
       <c r="W29">
-        <v>824.3725758992462</v>
+        <v>499.7552234475213</v>
+      </c>
+      <c r="X29">
+        <v>1558.361130169412</v>
+      </c>
+      <c r="Y29">
+        <v>799.7175932156176</v>
+      </c>
+      <c r="Z29">
+        <v>475.1002407638928</v>
+      </c>
+      <c r="AA29">
+        <v>1533.706147485783</v>
+      </c>
+      <c r="AB29">
+        <v>12.86440677966102</v>
       </c>
     </row>
     <row r="30">
@@ -2546,17 +3075,35 @@
       <c r="R30">
         <v>-22.93640367452804</v>
       </c>
+      <c r="S30">
+        <v>686.5262758335965</v>
+      </c>
       <c r="T30">
-        <v>686.5262758335965</v>
+        <v>171.6315689583991</v>
       </c>
       <c r="U30">
-        <v>171.6315689583991</v>
+        <v>1830.736735556257</v>
       </c>
       <c r="V30">
-        <v>1830.736735556257</v>
+        <v>1056.545682643785</v>
       </c>
       <c r="W30">
-        <v>1056.545682643785</v>
+        <v>550.7299688897549</v>
+      </c>
+      <c r="X30">
+        <v>2191.677149245278</v>
+      </c>
+      <c r="Y30">
+        <v>1028.33528313792</v>
+      </c>
+      <c r="Z30">
+        <v>522.5195693838896</v>
+      </c>
+      <c r="AA30">
+        <v>2163.466749739413</v>
+      </c>
+      <c r="AB30">
+        <v>6.135593220338983</v>
       </c>
     </row>
     <row r="31">
@@ -2618,17 +3165,35 @@
       <c r="R31">
         <v>-132.4114092948746</v>
       </c>
+      <c r="S31">
+        <v>-348.1786362533473</v>
+      </c>
       <c r="T31">
-        <v>-348.1786362533473</v>
+        <v>-87.04465906333684</v>
       </c>
       <c r="U31">
-        <v>-87.04465906333684</v>
+        <v>-928.4763633422596</v>
       </c>
       <c r="V31">
-        <v>-928.4763633422596</v>
+        <v>-317.3432051086431</v>
       </c>
       <c r="W31">
-        <v>-317.3432051086431</v>
+        <v>-3.796378406078077</v>
+      </c>
+      <c r="X31">
+        <v>-950.05378171011</v>
+      </c>
+      <c r="Y31">
+        <v>-328.6484831664309</v>
+      </c>
+      <c r="Z31">
+        <v>-15.10165646386598</v>
+      </c>
+      <c r="AA31">
+        <v>-961.3590597678979</v>
+      </c>
+      <c r="AB31">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -2690,17 +3255,35 @@
       <c r="R32">
         <v>-32.7771120167408</v>
       </c>
+      <c r="S32">
+        <v>285.0303606961218</v>
+      </c>
       <c r="T32">
-        <v>285.0303606961218</v>
+        <v>71.25759017403045</v>
       </c>
       <c r="U32">
-        <v>71.25759017403045</v>
+        <v>760.0809618563248</v>
       </c>
       <c r="V32">
-        <v>760.0809618563248</v>
+        <v>625.8505085155165</v>
       </c>
       <c r="W32">
-        <v>625.8505085155165</v>
+        <v>425.0520115000517</v>
+      </c>
+      <c r="X32">
+        <v>1087.926836169093</v>
+      </c>
+      <c r="Y32">
+        <v>595.5769970393969</v>
+      </c>
+      <c r="Z32">
+        <v>394.7785000239322</v>
+      </c>
+      <c r="AA32">
+        <v>1057.653324692973</v>
+      </c>
+      <c r="AB32">
+        <v>6</v>
       </c>
     </row>
     <row r="33">
@@ -2762,17 +3345,35 @@
       <c r="R33">
         <v>-99.32213809590436</v>
       </c>
+      <c r="S33">
+        <v>-245.2723622574324</v>
+      </c>
       <c r="T33">
-        <v>-245.2723622574324</v>
+        <v>-61.31809056435809</v>
       </c>
       <c r="U33">
-        <v>-61.31809056435809</v>
+        <v>-654.0596326864863</v>
       </c>
       <c r="V33">
-        <v>-654.0596326864863</v>
+        <v>149.4526768719323</v>
       </c>
       <c r="W33">
-        <v>149.4526768719323</v>
+        <v>372.7219615613021</v>
+      </c>
+      <c r="X33">
+        <v>-298.6496065534171</v>
+      </c>
+      <c r="Y33">
+        <v>44.14236615847625</v>
+      </c>
+      <c r="Z33">
+        <v>267.411650847846</v>
+      </c>
+      <c r="AA33">
+        <v>-403.9599172668732</v>
+      </c>
+      <c r="AB33">
+        <v>0.7333333333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2834,17 +3435,35 @@
       <c r="R34">
         <v>-33.75375027892549</v>
       </c>
+      <c r="S34">
+        <v>-71.83156791000187</v>
+      </c>
       <c r="T34">
-        <v>-71.83156791000187</v>
+        <v>-17.95789197750047</v>
       </c>
       <c r="U34">
-        <v>-17.95789197750047</v>
+        <v>-191.550847760005</v>
       </c>
       <c r="V34">
-        <v>-191.550847760005</v>
+        <v>449.2467190357018</v>
       </c>
       <c r="W34">
-        <v>449.2467190357018</v>
+        <v>516.4812544536112</v>
+      </c>
+      <c r="X34">
+        <v>316.1665797002906</v>
+      </c>
+      <c r="Y34">
+        <v>415.365685663722</v>
+      </c>
+      <c r="Z34">
+        <v>482.6002210816314</v>
+      </c>
+      <c r="AA34">
+        <v>282.2855463283109</v>
+      </c>
+      <c r="AB34">
+        <v>3.610169491525424</v>
       </c>
     </row>
     <row r="35">
@@ -2906,17 +3525,35 @@
       <c r="R35">
         <v>-69.76600477359052</v>
       </c>
+      <c r="S35">
+        <v>715.1119955715096</v>
+      </c>
       <c r="T35">
-        <v>715.1119955715096</v>
+        <v>178.7779988928774</v>
       </c>
       <c r="U35">
-        <v>178.7779988928774</v>
+        <v>1906.965321524026</v>
       </c>
       <c r="V35">
-        <v>1906.965321524026</v>
+        <v>1004.275094602528</v>
       </c>
       <c r="W35">
-        <v>1004.275094602528</v>
+        <v>495.5568081467759</v>
+      </c>
+      <c r="X35">
+        <v>2168.512710332165</v>
+      </c>
+      <c r="Y35">
+        <v>971.2547734051061</v>
+      </c>
+      <c r="Z35">
+        <v>462.5364869493534</v>
+      </c>
+      <c r="AA35">
+        <v>2135.492389134743</v>
+      </c>
+      <c r="AB35">
+        <v>6.220338983050848</v>
       </c>
     </row>
     <row r="36">
@@ -2978,17 +3615,35 @@
       <c r="R36">
         <v>-27.22953876710327</v>
       </c>
+      <c r="S36">
+        <v>799.9688724580296</v>
+      </c>
       <c r="T36">
-        <v>799.9688724580296</v>
+        <v>199.9922181145074</v>
       </c>
       <c r="U36">
-        <v>199.9922181145074</v>
+        <v>2133.250326554746</v>
       </c>
       <c r="V36">
-        <v>2133.250326554746</v>
+        <v>1186.53682919157</v>
       </c>
       <c r="W36">
-        <v>1186.53682919157</v>
+        <v>597.3385339433598</v>
+      </c>
+      <c r="X36">
+        <v>2509.039924192975</v>
+      </c>
+      <c r="Y36">
+        <v>1159.982421763237</v>
+      </c>
+      <c r="Z36">
+        <v>570.7841265150265</v>
+      </c>
+      <c r="AA36">
+        <v>2482.485516764642</v>
+      </c>
+      <c r="AB36">
+        <v>11.2</v>
       </c>
     </row>
     <row r="37">
@@ -3050,17 +3705,35 @@
       <c r="R37">
         <v>-18.58141926439271</v>
       </c>
+      <c r="S37">
+        <v>115.1339448338881</v>
+      </c>
       <c r="T37">
-        <v>115.1339448338881</v>
+        <v>28.78348620847201</v>
       </c>
       <c r="U37">
-        <v>28.78348620847201</v>
+        <v>307.0238528903681</v>
       </c>
       <c r="V37">
-        <v>307.0238528903681</v>
+        <v>282.9823514673414</v>
       </c>
       <c r="W37">
-        <v>282.9823514673414</v>
+        <v>203.9870379674142</v>
+      </c>
+      <c r="X37">
+        <v>467.5171143983328</v>
+      </c>
+      <c r="Y37">
+        <v>269.402918366946</v>
+      </c>
+      <c r="Z37">
+        <v>190.4076048670188</v>
+      </c>
+      <c r="AA37">
+        <v>453.9376812979373</v>
+      </c>
+      <c r="AB37">
+        <v>2</v>
       </c>
     </row>
     <row r="38">
@@ -3122,17 +3795,35 @@
       <c r="R38">
         <v>-57.70377317826512</v>
       </c>
+      <c r="S38">
+        <v>-391.0246525627841</v>
+      </c>
       <c r="T38">
-        <v>-391.0246525627841</v>
+        <v>-97.75616314069602</v>
       </c>
       <c r="U38">
-        <v>-97.75616314069602</v>
+        <v>-1042.732406834091</v>
       </c>
       <c r="V38">
-        <v>-1042.732406834091</v>
+        <v>-249.9471891329695</v>
       </c>
       <c r="W38">
-        <v>-249.9471891329695</v>
+        <v>66.16237717218181</v>
+      </c>
+      <c r="X38">
+        <v>-924.4960202873397</v>
+      </c>
+      <c r="Y38">
+        <v>-268.3901425190508</v>
+      </c>
+      <c r="Z38">
+        <v>47.71942378610061</v>
+      </c>
+      <c r="AA38">
+        <v>-942.9389736734208</v>
+      </c>
+      <c r="AB38">
+        <v>1.88135593220339</v>
       </c>
     </row>
     <row r="39">
@@ -3194,17 +3885,35 @@
       <c r="R39">
         <v>-37.82831323651127</v>
       </c>
+      <c r="S39">
+        <v>-273.0250565140611</v>
+      </c>
       <c r="T39">
-        <v>-273.0250565140611</v>
+        <v>-68.25626412851528</v>
       </c>
       <c r="U39">
-        <v>-68.25626412851528</v>
+        <v>-728.0668173708297</v>
       </c>
       <c r="V39">
-        <v>-728.0668173708297</v>
+        <v>272.2734425938952</v>
       </c>
       <c r="W39">
-        <v>272.2734425938952</v>
+        <v>492.0159423022267</v>
+      </c>
+      <c r="X39">
+        <v>-197.742025585659</v>
+      </c>
+      <c r="Y39">
+        <v>230.0257972189942</v>
+      </c>
+      <c r="Z39">
+        <v>449.7682969273257</v>
+      </c>
+      <c r="AA39">
+        <v>-239.98967096056</v>
+      </c>
+      <c r="AB39">
+        <v>6.915254237288136</v>
       </c>
     </row>
     <row r="40">
@@ -3266,17 +3975,35 @@
       <c r="R40">
         <v>-88.29875926621034</v>
       </c>
+      <c r="S40">
+        <v>204.5507074525101</v>
+      </c>
       <c r="T40">
-        <v>204.5507074525101</v>
+        <v>51.13767686312753</v>
       </c>
       <c r="U40">
-        <v>51.13767686312753</v>
+        <v>545.4685532066936</v>
       </c>
       <c r="V40">
-        <v>545.4685532066936</v>
+        <v>726.7926710539176</v>
       </c>
       <c r="W40">
-        <v>726.7926710539176</v>
+        <v>608.3312326740765</v>
+      </c>
+      <c r="X40">
+        <v>1032.75892459856</v>
+      </c>
+      <c r="Y40">
+        <v>678.9956463740091</v>
+      </c>
+      <c r="Z40">
+        <v>560.534207994168</v>
+      </c>
+      <c r="AA40">
+        <v>984.9618999186509</v>
+      </c>
+      <c r="AB40">
+        <v>11.22033898305085</v>
       </c>
     </row>
     <row r="41">
@@ -3338,17 +4065,35 @@
       <c r="R41">
         <v>-31.9976583991754</v>
       </c>
+      <c r="S41">
+        <v>-966.0429212020487</v>
+      </c>
       <c r="T41">
-        <v>-966.0429212020487</v>
+        <v>-241.5107303005122</v>
       </c>
       <c r="U41">
-        <v>-241.5107303005122</v>
+        <v>-2576.114456538796</v>
       </c>
       <c r="V41">
-        <v>-2576.114456538796</v>
+        <v>-720.5023570183444</v>
       </c>
       <c r="W41">
-        <v>-720.5023570183444</v>
+        <v>16.69557366619898</v>
+      </c>
+      <c r="X41">
+        <v>-2343.239632138098</v>
+      </c>
+      <c r="Y41">
+        <v>-747.1229371569049</v>
+      </c>
+      <c r="Z41">
+        <v>-9.925006472361559</v>
+      </c>
+      <c r="AA41">
+        <v>-2369.860212276659</v>
+      </c>
+      <c r="AB41">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -3410,17 +4155,35 @@
       <c r="R42">
         <v>-66.6095139583979</v>
       </c>
+      <c r="S42">
+        <v>-1141.569156945336</v>
+      </c>
       <c r="T42">
-        <v>-1141.569156945336</v>
+        <v>-285.3922892363341</v>
       </c>
       <c r="U42">
-        <v>-285.3922892363341</v>
+        <v>-3044.184418520897</v>
       </c>
       <c r="V42">
-        <v>-3044.184418520897</v>
+        <v>-1004.984809253795</v>
       </c>
       <c r="W42">
-        <v>-1004.984809253795</v>
+        <v>-122.4416756029266</v>
+      </c>
+      <c r="X42">
+        <v>-2933.966336771221</v>
+      </c>
+      <c r="Y42">
+        <v>-1057.312660164985</v>
+      </c>
+      <c r="Z42">
+        <v>-174.7695265141175</v>
+      </c>
+      <c r="AA42">
+        <v>-2986.294187682412</v>
+      </c>
+      <c r="AB42">
+        <v>1.932203389830508</v>
       </c>
     </row>
     <row r="43">
@@ -3482,17 +4245,35 @@
       <c r="R43">
         <v>-43.57228032095942</v>
       </c>
+      <c r="S43">
+        <v>-1624.929458919247</v>
+      </c>
       <c r="T43">
-        <v>-1624.929458919247</v>
+        <v>-406.2323647298118</v>
       </c>
       <c r="U43">
-        <v>-406.2323647298118</v>
+        <v>-4333.14522378466</v>
       </c>
       <c r="V43">
-        <v>-4333.14522378466</v>
+        <v>-1359.242743335986</v>
       </c>
       <c r="W43">
-        <v>-1359.242743335986</v>
+        <v>-123.2982881861705</v>
+      </c>
+      <c r="X43">
+        <v>-4084.705869161778</v>
+      </c>
+      <c r="Y43">
+        <v>-1415.440416557498</v>
+      </c>
+      <c r="Z43">
+        <v>-179.4959614076831</v>
+      </c>
+      <c r="AA43">
+        <v>-4140.90354238329</v>
+      </c>
+      <c r="AB43">
+        <v>3.491525423728814</v>
       </c>
     </row>
     <row r="44">
@@ -3554,17 +4335,35 @@
       <c r="R44">
         <v>-23.5983827663694</v>
       </c>
+      <c r="S44">
+        <v>-931.5429266587793</v>
+      </c>
       <c r="T44">
-        <v>-931.5429266587793</v>
+        <v>-232.8857316646948</v>
       </c>
       <c r="U44">
-        <v>-232.8857316646948</v>
+        <v>-2484.114471090078</v>
       </c>
       <c r="V44">
-        <v>-2484.114471090078</v>
+        <v>-532.5656404606669</v>
       </c>
       <c r="W44">
-        <v>-532.5656404606669</v>
+        <v>175.4325810451055</v>
+      </c>
+      <c r="X44">
+        <v>-2094.478211403653</v>
+      </c>
+      <c r="Y44">
+        <v>-563.6874830146545</v>
+      </c>
+      <c r="Z44">
+        <v>144.3107384911179</v>
+      </c>
+      <c r="AA44">
+        <v>-2125.600053957641</v>
+      </c>
+      <c r="AB44">
+        <v>6.35593220338983</v>
       </c>
     </row>
     <row r="45">
@@ -3626,17 +4425,35 @@
       <c r="R45">
         <v>-35.26445651144341</v>
       </c>
+      <c r="S45">
+        <v>-28.55696837950058</v>
+      </c>
       <c r="T45">
-        <v>-28.55696837950058</v>
+        <v>-7.139242094875145</v>
       </c>
       <c r="U45">
-        <v>-7.139242094875145</v>
+        <v>-76.15191567866822</v>
       </c>
       <c r="V45">
-        <v>-76.15191567866822</v>
+        <v>524.8476553689155</v>
       </c>
       <c r="W45">
-        <v>524.8476553689155</v>
+        <v>560.224229022654</v>
+      </c>
+      <c r="X45">
+        <v>463.2938607006349</v>
+      </c>
+      <c r="Y45">
+        <v>479.3620370902144</v>
+      </c>
+      <c r="Z45">
+        <v>514.7386107439528</v>
+      </c>
+      <c r="AA45">
+        <v>417.8082424219337</v>
+      </c>
+      <c r="AB45">
+        <v>5.491525423728813</v>
       </c>
     </row>
     <row r="46">
@@ -3698,17 +4515,35 @@
       <c r="R46">
         <v>-17.35655505192626</v>
       </c>
+      <c r="S46">
+        <v>-794.2045027091767</v>
+      </c>
       <c r="T46">
-        <v>-794.2045027091767</v>
+        <v>-198.5511256772942</v>
       </c>
       <c r="U46">
-        <v>-198.5511256772942</v>
+        <v>-2117.878673891138</v>
       </c>
       <c r="V46">
-        <v>-2117.878673891138</v>
+        <v>-525.2320455214378</v>
       </c>
       <c r="W46">
-        <v>-525.2320455214378</v>
+        <v>77.29163455183217</v>
+      </c>
+      <c r="X46">
+        <v>-1855.776519744787</v>
+      </c>
+      <c r="Y46">
+        <v>-563.1657076070233</v>
+      </c>
+      <c r="Z46">
+        <v>39.35797246624679</v>
+      </c>
+      <c r="AA46">
+        <v>-1893.710181830372</v>
+      </c>
+      <c r="AB46">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -3770,17 +4605,35 @@
       <c r="R47">
         <v>-29.66221983874401</v>
       </c>
+      <c r="S47">
+        <v>-13.28549215938822</v>
+      </c>
       <c r="T47">
-        <v>-13.28549215938822</v>
+        <v>-3.321373039847054</v>
       </c>
       <c r="U47">
-        <v>-3.321373039847054</v>
+        <v>-35.42797909170191</v>
       </c>
       <c r="V47">
-        <v>-35.42797909170191</v>
+        <v>575.0969783561879</v>
       </c>
       <c r="W47">
-        <v>575.0969783561879</v>
+        <v>596.8023928285653</v>
+      </c>
+      <c r="X47">
+        <v>541.2131960710381</v>
+      </c>
+      <c r="Y47">
+        <v>516.9012879491287</v>
+      </c>
+      <c r="Z47">
+        <v>538.606702421506</v>
+      </c>
+      <c r="AA47">
+        <v>483.0175056639788</v>
+      </c>
+      <c r="AB47">
+        <v>6.203389830508475</v>
       </c>
     </row>
     <row r="48">
@@ -3842,17 +4695,35 @@
       <c r="R48">
         <v>-25.9084799374745</v>
       </c>
+      <c r="S48">
+        <v>-907.9343167996072</v>
+      </c>
       <c r="T48">
-        <v>-907.9343167996072</v>
+        <v>-226.9835791999018</v>
       </c>
       <c r="U48">
-        <v>-226.9835791999018</v>
+        <v>-2421.158178132286</v>
       </c>
       <c r="V48">
-        <v>-2421.158178132286</v>
+        <v>-660.1522980368836</v>
       </c>
       <c r="W48">
-        <v>-660.1522980368836</v>
+        <v>31.05387953807224</v>
+      </c>
+      <c r="X48">
+        <v>-2183.631599344813</v>
+      </c>
+      <c r="Y48">
+        <v>-697.9962543978402</v>
+      </c>
+      <c r="Z48">
+        <v>-6.790076822884373</v>
+      </c>
+      <c r="AA48">
+        <v>-2221.475555705769</v>
+      </c>
+      <c r="AB48">
+        <v>1.864406779661017</v>
       </c>
     </row>
     <row r="49">
@@ -3914,17 +4785,35 @@
       <c r="R49">
         <v>-19.43462453174192</v>
       </c>
+      <c r="S49">
+        <v>-13.44608419750229</v>
+      </c>
       <c r="T49">
-        <v>-13.44608419750229</v>
+        <v>-3.361521049375571</v>
       </c>
       <c r="U49">
-        <v>-3.361521049375571</v>
+        <v>-35.85622452667276</v>
       </c>
       <c r="V49">
-        <v>-35.85622452667276</v>
+        <v>448.3065100927043</v>
       </c>
       <c r="W49">
-        <v>448.3065100927043</v>
+        <v>466.0839454513122</v>
+      </c>
+      <c r="X49">
+        <v>418.2034975530526</v>
+      </c>
+      <c r="Y49">
+        <v>431.0169806587588</v>
+      </c>
+      <c r="Z49">
+        <v>448.7944160173667</v>
+      </c>
+      <c r="AA49">
+        <v>400.9139681191072</v>
+      </c>
+      <c r="AB49">
+        <v>11.5</v>
       </c>
     </row>
     <row r="50">
@@ -3986,17 +4875,35 @@
       <c r="R50">
         <v>-28.01301462364787</v>
       </c>
+      <c r="S50">
+        <v>38.77324499785593</v>
+      </c>
       <c r="T50">
-        <v>38.77324499785593</v>
+        <v>9.693311249463981</v>
       </c>
       <c r="U50">
-        <v>9.693311249463981</v>
+        <v>103.3953199942825</v>
       </c>
       <c r="V50">
-        <v>103.3953199942825</v>
+        <v>378.3542944840665</v>
       </c>
       <c r="W50">
-        <v>378.3542944840665</v>
+        <v>360.3628456908685</v>
+      </c>
+      <c r="X50">
+        <v>431.8878845252991</v>
+      </c>
+      <c r="Y50">
+        <v>363.1882784791776</v>
+      </c>
+      <c r="Z50">
+        <v>345.1968296859796</v>
+      </c>
+      <c r="AA50">
+        <v>416.7218685204102</v>
+      </c>
+      <c r="AB50">
+        <v>3.254237288135593</v>
       </c>
     </row>
     <row r="51">
@@ -4058,17 +4965,35 @@
       <c r="R51">
         <v>-192.9124417585077</v>
       </c>
+      <c r="S51">
+        <v>-459.991635634027</v>
+      </c>
       <c r="T51">
-        <v>-459.991635634027</v>
+        <v>-114.9979089085068</v>
       </c>
       <c r="U51">
-        <v>-114.9979089085068</v>
+        <v>-1226.644361690739</v>
       </c>
       <c r="V51">
-        <v>-1226.644361690739</v>
+        <v>-439.1394011764789</v>
       </c>
       <c r="W51">
-        <v>-439.1394011764789</v>
+        <v>-17.78449958821597</v>
+      </c>
+      <c r="X51">
+        <v>-1282.153302095933</v>
+      </c>
+      <c r="Y51">
+        <v>-467.2487512155525</v>
+      </c>
+      <c r="Z51">
+        <v>-45.89384962728975</v>
+      </c>
+      <c r="AA51">
+        <v>-1310.262652135007</v>
+      </c>
+      <c r="AB51">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -4130,17 +5055,35 @@
       <c r="R52">
         <v>-27.48984268260899</v>
       </c>
+      <c r="S52">
+        <v>-531.4328454065576</v>
+      </c>
       <c r="T52">
-        <v>-531.4328454065576</v>
+        <v>-132.8582113516394</v>
       </c>
       <c r="U52">
-        <v>-132.8582113516394</v>
+        <v>-1417.154254417487</v>
       </c>
       <c r="V52">
-        <v>-1417.154254417487</v>
+        <v>-148.524553898246</v>
       </c>
       <c r="W52">
-        <v>-148.524553898246</v>
+        <v>260.9314762185383</v>
+      </c>
+      <c r="X52">
+        <v>-1045.127358971041</v>
+      </c>
+      <c r="Y52">
+        <v>-170.4165242918114</v>
+      </c>
+      <c r="Z52">
+        <v>239.0395058249728</v>
+      </c>
+      <c r="AA52">
+        <v>-1067.019329364607</v>
+      </c>
+      <c r="AB52">
+        <v>3.033898305084746</v>
       </c>
     </row>
     <row r="53">
@@ -4202,17 +5145,35 @@
       <c r="R53">
         <v>-39.04530378209561</v>
       </c>
+      <c r="S53">
+        <v>-203.5334048808638</v>
+      </c>
       <c r="T53">
-        <v>-203.5334048808638</v>
+        <v>-50.88335122021595</v>
       </c>
       <c r="U53">
-        <v>-50.88335122021595</v>
+        <v>-542.7557463489701</v>
       </c>
       <c r="V53">
-        <v>-542.7557463489701</v>
+        <v>372.0900869812113</v>
       </c>
       <c r="W53">
-        <v>372.0900869812113</v>
+        <v>540.1955733889387</v>
+      </c>
+      <c r="X53">
+        <v>17.41231276602548</v>
+      </c>
+      <c r="Y53">
+        <v>318.56705918585</v>
+      </c>
+      <c r="Z53">
+        <v>486.6725455935774</v>
+      </c>
+      <c r="AA53">
+        <v>-36.11071502933578</v>
+      </c>
+      <c r="AB53">
+        <v>10.33898305084746</v>
       </c>
     </row>
     <row r="54">
@@ -4274,17 +5235,35 @@
       <c r="R54">
         <v>-81.71405011370113</v>
       </c>
+      <c r="S54">
+        <v>-513.3567931933326</v>
+      </c>
       <c r="T54">
-        <v>-513.3567931933326</v>
+        <v>-128.3391982983331</v>
       </c>
       <c r="U54">
-        <v>-128.3391982983331</v>
+        <v>-1368.951448515553</v>
       </c>
       <c r="V54">
-        <v>-1368.951448515553</v>
+        <v>-487.976452147667</v>
       </c>
       <c r="W54">
-        <v>-487.976452147667</v>
+        <v>-70.61371241599413</v>
+      </c>
+      <c r="X54">
+        <v>-1375.916252306561</v>
+      </c>
+      <c r="Y54">
+        <v>-516.868643012019</v>
+      </c>
+      <c r="Z54">
+        <v>-99.50590328034613</v>
+      </c>
+      <c r="AA54">
+        <v>-1404.808443170913</v>
+      </c>
+      <c r="AB54">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -4346,17 +5325,35 @@
       <c r="R55">
         <v>-40.86534077375143</v>
       </c>
+      <c r="S55">
+        <v>-847.4048581032467</v>
+      </c>
       <c r="T55">
-        <v>-847.4048581032467</v>
+        <v>-211.8512145258117</v>
       </c>
       <c r="U55">
-        <v>-211.8512145258117</v>
+        <v>-2259.746288275325</v>
       </c>
       <c r="V55">
-        <v>-2259.746288275325</v>
+        <v>-721.7365338639902</v>
       </c>
       <c r="W55">
-        <v>-721.7365338639902</v>
+        <v>-70.00702623027863</v>
+      </c>
+      <c r="X55">
+        <v>-2150.253828092345</v>
+      </c>
+      <c r="Y55">
+        <v>-736.5943050616972</v>
+      </c>
+      <c r="Z55">
+        <v>-84.86479742798562</v>
+      </c>
+      <c r="AA55">
+        <v>-2165.111599290052</v>
+      </c>
+      <c r="AB55">
+        <v>1.983050847457627</v>
       </c>
     </row>
     <row r="56">
@@ -4418,17 +5415,35 @@
       <c r="R56">
         <v>-84.48347779409866</v>
       </c>
+      <c r="S56">
+        <v>-639.6921167376527</v>
+      </c>
       <c r="T56">
-        <v>-639.6921167376527</v>
+        <v>-159.9230291844132</v>
       </c>
       <c r="U56">
-        <v>-159.9230291844132</v>
+        <v>-1705.84564463374</v>
       </c>
       <c r="V56">
-        <v>-1705.84564463374</v>
+        <v>-171.6367584212563</v>
       </c>
       <c r="W56">
-        <v>-171.6367584212563</v>
+        <v>341.5737057588138</v>
+      </c>
+      <c r="X56">
+        <v>-1271.231662944174</v>
+      </c>
+      <c r="Y56">
+        <v>-206.1963833853746</v>
+      </c>
+      <c r="Z56">
+        <v>307.0140807946956</v>
+      </c>
+      <c r="AA56">
+        <v>-1305.791287908293</v>
+      </c>
+      <c r="AB56">
+        <v>5.186440677966102</v>
       </c>
     </row>
     <row r="57">
@@ -4490,17 +5505,35 @@
       <c r="R57">
         <v>-191.2174984961702</v>
       </c>
+      <c r="S57">
+        <v>-262.5861493309494</v>
+      </c>
       <c r="T57">
-        <v>-262.5861493309494</v>
+        <v>-65.64653733273735</v>
       </c>
       <c r="U57">
-        <v>-65.64653733273735</v>
+        <v>-700.2297315491984</v>
       </c>
       <c r="V57">
-        <v>-700.2297315491984</v>
+        <v>-120.9078985152807</v>
       </c>
       <c r="W57">
-        <v>-120.9078985152807</v>
+        <v>151.721973304332</v>
+      </c>
+      <c r="X57">
+        <v>-634.2417405549304</v>
+      </c>
+      <c r="Y57">
+        <v>-178.5915714805676</v>
+      </c>
+      <c r="Z57">
+        <v>94.03830033904518</v>
+      </c>
+      <c r="AA57">
+        <v>-691.9254135202173</v>
+      </c>
+      <c r="AB57">
+        <v>1.983050847457627</v>
       </c>
     </row>
     <row r="58">
@@ -4562,17 +5595,35 @@
       <c r="R58">
         <v>-40.92084729343487</v>
       </c>
+      <c r="S58">
+        <v>-30.98620230848367</v>
+      </c>
       <c r="T58">
-        <v>-30.98620230848367</v>
+        <v>-7.746550577120918</v>
       </c>
       <c r="U58">
-        <v>-7.746550577120918</v>
+        <v>-82.62987282262313</v>
       </c>
       <c r="V58">
-        <v>-82.62987282262313</v>
+        <v>525.2162277796139</v>
       </c>
       <c r="W58">
-        <v>525.2162277796139</v>
+        <v>564.6537148979612</v>
+      </c>
+      <c r="X58">
+        <v>457.3747218784898</v>
+      </c>
+      <c r="Y58">
+        <v>479.1199025310208</v>
+      </c>
+      <c r="Z58">
+        <v>518.5573896493681</v>
+      </c>
+      <c r="AA58">
+        <v>411.2783966298967</v>
+      </c>
+      <c r="AB58">
+        <v>12.3</v>
       </c>
     </row>
     <row r="59">
@@ -4634,17 +5685,35 @@
       <c r="R59">
         <v>-28.55390149364721</v>
       </c>
+      <c r="S59">
+        <v>198.2104816727272</v>
+      </c>
       <c r="T59">
-        <v>198.2104816727272</v>
+        <v>49.55262041818181</v>
       </c>
       <c r="U59">
-        <v>49.55262041818181</v>
+        <v>528.561284460606</v>
       </c>
       <c r="V59">
-        <v>528.561284460606</v>
+        <v>580.4545005526619</v>
       </c>
       <c r="W59">
-        <v>580.4545005526619</v>
+        <v>443.0992253060186</v>
+      </c>
+      <c r="X59">
+        <v>899.5027173326387</v>
+      </c>
+      <c r="Y59">
+        <v>531.1908363692988</v>
+      </c>
+      <c r="Z59">
+        <v>393.8355611226555</v>
+      </c>
+      <c r="AA59">
+        <v>850.2390531492756</v>
+      </c>
+      <c r="AB59">
+        <v>3.416666666666667</v>
       </c>
     </row>
     <row r="60">
@@ -4706,17 +5775,35 @@
       <c r="R60">
         <v>-46.53095406663628</v>
       </c>
+      <c r="S60">
+        <v>150.8143772717958</v>
+      </c>
       <c r="T60">
-        <v>150.8143772717958</v>
+        <v>37.70359431794895</v>
       </c>
       <c r="U60">
-        <v>37.70359431794895</v>
+        <v>402.1716727247888</v>
       </c>
       <c r="V60">
-        <v>402.1716727247888</v>
+        <v>737.7854905920595</v>
       </c>
       <c r="W60">
-        <v>737.7854905920595</v>
+        <v>643.0932102895896</v>
+      </c>
+      <c r="X60">
+        <v>970.7242833936757</v>
+      </c>
+      <c r="Y60">
+        <v>717.3337827361231</v>
+      </c>
+      <c r="Z60">
+        <v>622.6415024336532</v>
+      </c>
+      <c r="AA60">
+        <v>950.2725755377392</v>
+      </c>
+      <c r="AB60">
+        <v>11.28813559322034</v>
       </c>
     </row>
     <row r="61">
@@ -4778,17 +5865,35 @@
       <c r="R61">
         <v>-17.32788108365847</v>
       </c>
+      <c r="S61">
+        <v>841.474237757583</v>
+      </c>
       <c r="T61">
-        <v>841.474237757583</v>
+        <v>210.3685594393957</v>
       </c>
       <c r="U61">
-        <v>210.3685594393957</v>
+        <v>2243.931300686888</v>
       </c>
       <c r="V61">
-        <v>2243.931300686888</v>
+        <v>1181.254353969848</v>
       </c>
       <c r="W61">
-        <v>1181.254353969848</v>
+        <v>557.0076285806088</v>
+      </c>
+      <c r="X61">
+        <v>2576.852463970205</v>
+      </c>
+      <c r="Y61">
+        <v>1167.722676300931</v>
+      </c>
+      <c r="Z61">
+        <v>543.4759509116923</v>
+      </c>
+      <c r="AA61">
+        <v>2563.320786301288</v>
+      </c>
+      <c r="AB61">
+        <v>13</v>
       </c>
     </row>
     <row r="62">
@@ -4850,17 +5955,35 @@
       <c r="R62">
         <v>-31.01756894557587</v>
       </c>
+      <c r="S62">
+        <v>-587.0267300596598</v>
+      </c>
       <c r="T62">
-        <v>-587.0267300596598</v>
+        <v>-146.756682514915</v>
       </c>
       <c r="U62">
-        <v>-146.756682514915</v>
+        <v>-1565.404613492426</v>
       </c>
       <c r="V62">
-        <v>-1565.404613492426</v>
+        <v>-601.6420896740709</v>
       </c>
       <c r="W62">
-        <v>-601.6420896740709</v>
+        <v>-149.0942544217023</v>
+      </c>
+      <c r="X62">
+        <v>-1592.297760814461</v>
+      </c>
+      <c r="Y62">
+        <v>-602.4638077989824</v>
+      </c>
+      <c r="Z62">
+        <v>-149.9159725466138</v>
+      </c>
+      <c r="AA62">
+        <v>-1593.119478939373</v>
+      </c>
+      <c r="AB62">
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="63">
@@ -4922,17 +6045,35 @@
       <c r="R63">
         <v>-109.0449560586357</v>
       </c>
+      <c r="S63">
+        <v>-1087.409657566273</v>
+      </c>
       <c r="T63">
-        <v>-1087.409657566273</v>
+        <v>-271.8524143915683</v>
       </c>
       <c r="U63">
-        <v>-271.8524143915683</v>
+        <v>-2899.759086843396</v>
       </c>
       <c r="V63">
-        <v>-2899.759086843396</v>
+        <v>-815.3844434125592</v>
       </c>
       <c r="W63">
-        <v>-815.3844434125592</v>
+        <v>43.33642820202243</v>
+      </c>
+      <c r="X63">
+        <v>-2670.897501129558</v>
+      </c>
+      <c r="Y63">
+        <v>-834.7163274478626</v>
+      </c>
+      <c r="Z63">
+        <v>24.00454416671874</v>
+      </c>
+      <c r="AA63">
+        <v>-2690.229385164862</v>
+      </c>
+      <c r="AB63">
+        <v>2.95</v>
       </c>
     </row>
     <row r="64">
@@ -4994,17 +6135,35 @@
       <c r="R64">
         <v>-41.26914297593793</v>
       </c>
+      <c r="S64">
+        <v>858.0909074004417</v>
+      </c>
       <c r="T64">
-        <v>858.0909074004417</v>
+        <v>214.5227268501104</v>
       </c>
       <c r="U64">
-        <v>214.5227268501104</v>
+        <v>2288.242419734511</v>
       </c>
       <c r="V64">
-        <v>2288.242419734511</v>
+        <v>1003.581557869952</v>
       </c>
       <c r="W64">
-        <v>1003.581557869952</v>
+        <v>376.3490797475959</v>
+      </c>
+      <c r="X64">
+        <v>2417.397367776045</v>
+      </c>
+      <c r="Y64">
+        <v>995.4751110419594</v>
+      </c>
+      <c r="Z64">
+        <v>368.2426329196035</v>
+      </c>
+      <c r="AA64">
+        <v>2409.290920948053</v>
+      </c>
+      <c r="AB64">
+        <v>7.689655172413793</v>
       </c>
     </row>
     <row r="65">
@@ -5066,17 +6225,35 @@
       <c r="R65">
         <v>-149.8788793669305</v>
       </c>
+      <c r="S65">
+        <v>-103.0166085441775</v>
+      </c>
       <c r="T65">
-        <v>-103.0166085441775</v>
+        <v>-25.75415213604437</v>
       </c>
       <c r="U65">
-        <v>-25.75415213604437</v>
+        <v>-274.7109561178066</v>
       </c>
       <c r="V65">
-        <v>-274.7109561178066</v>
+        <v>-7.23298140177954</v>
       </c>
       <c r="W65">
-        <v>-7.23298140177954</v>
+        <v>129.3565314224302</v>
+      </c>
+      <c r="X65">
+        <v>-238.2543853914853</v>
+      </c>
+      <c r="Y65">
+        <v>-41.53900965587985</v>
+      </c>
+      <c r="Z65">
+        <v>95.05050316832994</v>
+      </c>
+      <c r="AA65">
+        <v>-272.5604136455856</v>
+      </c>
+      <c r="AB65">
+        <v>2.694915254237288</v>
       </c>
     </row>
     <row r="66">
@@ -5138,17 +6315,35 @@
       <c r="R66">
         <v>-37.57116634028481</v>
       </c>
+      <c r="S66">
+        <v>-350.5494967596808</v>
+      </c>
       <c r="T66">
-        <v>-350.5494967596808</v>
+        <v>-87.63737418992019</v>
       </c>
       <c r="U66">
-        <v>-87.63737418992019</v>
+        <v>-934.7986580258154</v>
       </c>
       <c r="V66">
-        <v>-934.7986580258154</v>
+        <v>-186.3947292709484</v>
       </c>
       <c r="W66">
-        <v>-186.3947292709484</v>
+        <v>91.38931330850824</v>
+      </c>
+      <c r="X66">
+        <v>-785.515810546779</v>
+      </c>
+      <c r="Y66">
+        <v>-197.0197132964836</v>
+      </c>
+      <c r="Z66">
+        <v>80.76432928297305</v>
+      </c>
+      <c r="AA66">
+        <v>-796.1407945723142</v>
+      </c>
+      <c r="AB66">
+        <v>6.677966101694915</v>
       </c>
     </row>
     <row r="67">
@@ -5210,17 +6405,35 @@
       <c r="R67">
         <v>-160.6197356223814</v>
       </c>
+      <c r="S67">
+        <v>-391.0487455847381</v>
+      </c>
       <c r="T67">
-        <v>-391.0487455847381</v>
+        <v>-97.76218639618452</v>
       </c>
       <c r="U67">
-        <v>-97.76218639618452</v>
+        <v>-1042.796654892635</v>
       </c>
       <c r="V67">
-        <v>-1042.796654892635</v>
+        <v>-365.1467769005856</v>
       </c>
       <c r="W67">
-        <v>-365.1467769005856</v>
+        <v>-8.281572361506065</v>
+      </c>
+      <c r="X67">
+        <v>-1080.473331559008</v>
+      </c>
+      <c r="Y67">
+        <v>-403.0909346856452</v>
+      </c>
+      <c r="Z67">
+        <v>-46.22573014656562</v>
+      </c>
+      <c r="AA67">
+        <v>-1118.417489344068</v>
+      </c>
+      <c r="AB67">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -5282,17 +6495,35 @@
       <c r="R68">
         <v>-21.87339065942142</v>
       </c>
+      <c r="S68">
+        <v>305.0015765069846</v>
+      </c>
       <c r="T68">
-        <v>305.0015765069846</v>
+        <v>76.25039412674616</v>
       </c>
       <c r="U68">
-        <v>76.25039412674616</v>
+        <v>813.337537351959</v>
       </c>
       <c r="V68">
-        <v>813.337537351959</v>
+        <v>673.6889168346786</v>
       </c>
       <c r="W68">
-        <v>673.6889168346786</v>
+        <v>453.5959515904611</v>
+      </c>
+      <c r="X68">
+        <v>1173.366660543632</v>
+      </c>
+      <c r="Y68">
+        <v>635.7517290549079</v>
+      </c>
+      <c r="Z68">
+        <v>415.6587638106904</v>
+      </c>
+      <c r="AA68">
+        <v>1135.429472763861</v>
+      </c>
+      <c r="AB68">
+        <v>6.610169491525424</v>
       </c>
     </row>
     <row r="69">
@@ -5354,17 +6585,35 @@
       <c r="R69">
         <v>-105.8550251002139</v>
       </c>
+      <c r="S69">
+        <v>-567.0975784374136</v>
+      </c>
       <c r="T69">
-        <v>-567.0975784374136</v>
+        <v>-141.7743946093534</v>
       </c>
       <c r="U69">
-        <v>-141.7743946093534</v>
+        <v>-1512.260209166436</v>
       </c>
       <c r="V69">
-        <v>-1512.260209166436</v>
+        <v>-163.3418305320671</v>
       </c>
       <c r="W69">
-        <v>-163.3418305320671</v>
+        <v>303.8823007314944</v>
+      </c>
+      <c r="X69">
+        <v>-1150.405408696591</v>
+      </c>
+      <c r="Y69">
+        <v>-207.9413614877236</v>
+      </c>
+      <c r="Z69">
+        <v>259.282769775838</v>
+      </c>
+      <c r="AA69">
+        <v>-1195.004939652247</v>
+      </c>
+      <c r="AB69">
+        <v>3.779661016949153</v>
       </c>
     </row>
     <row r="70">
@@ -5426,17 +6675,35 @@
       <c r="R70">
         <v>-37.38719156763692</v>
       </c>
+      <c r="S70">
+        <v>-505.8342403352136</v>
+      </c>
       <c r="T70">
-        <v>-505.8342403352136</v>
+        <v>-126.4585600838034</v>
       </c>
       <c r="U70">
-        <v>-126.4585600838034</v>
+        <v>-1348.89130756057</v>
       </c>
       <c r="V70">
-        <v>-1348.89130756057</v>
+        <v>-467.9859402922596</v>
       </c>
       <c r="W70">
-        <v>-467.9859402922596</v>
+        <v>-73.81116337865974</v>
+      </c>
+      <c r="X70">
+        <v>-1325.842104179806</v>
+      </c>
+      <c r="Y70">
+        <v>-487.9057667459891</v>
+      </c>
+      <c r="Z70">
+        <v>-93.7309898323893</v>
+      </c>
+      <c r="AA70">
+        <v>-1345.761930633535</v>
+      </c>
+      <c r="AB70">
+        <v>0.9833333333333333</v>
       </c>
     </row>
     <row r="71">
@@ -5498,17 +6765,35 @@
       <c r="R71">
         <v>-97.35207434179432</v>
       </c>
+      <c r="S71">
+        <v>-286.9955872458959</v>
+      </c>
       <c r="T71">
-        <v>-286.9955872458959</v>
+        <v>-71.74889681147397</v>
       </c>
       <c r="U71">
-        <v>-71.74889681147397</v>
+        <v>-765.3215659890557</v>
       </c>
       <c r="V71">
-        <v>-765.3215659890557</v>
+        <v>-198.7193698535926</v>
       </c>
       <c r="W71">
-        <v>-198.7193698535926</v>
+        <v>55.06251667445625</v>
+      </c>
+      <c r="X71">
+        <v>-715.5805446903794</v>
+      </c>
+      <c r="Y71">
+        <v>-240.5036130445687</v>
+      </c>
+      <c r="Z71">
+        <v>13.27827348348015</v>
+      </c>
+      <c r="AA71">
+        <v>-757.3647878813555</v>
+      </c>
+      <c r="AB71">
+        <v>0.9833333333333333</v>
       </c>
     </row>
     <row r="72">
@@ -5570,17 +6855,35 @@
       <c r="R72">
         <v>-24.8456317021995</v>
       </c>
+      <c r="S72">
+        <v>-290.4258767432515</v>
+      </c>
       <c r="T72">
-        <v>-290.4258767432515</v>
+        <v>-72.60646918581288</v>
       </c>
       <c r="U72">
-        <v>-72.60646918581288</v>
+        <v>-774.4690046486708</v>
       </c>
       <c r="V72">
-        <v>-774.4690046486708</v>
+        <v>-202.1198544544156</v>
       </c>
       <c r="W72">
-        <v>-202.1198544544156</v>
+        <v>25.53428231847705</v>
+      </c>
+      <c r="X72">
+        <v>-695.9977115752888</v>
+      </c>
+      <c r="Y72">
+        <v>-219.0974502870816</v>
+      </c>
+      <c r="Z72">
+        <v>8.556686485810985</v>
+      </c>
+      <c r="AA72">
+        <v>-712.9753074079548</v>
+      </c>
+      <c r="AB72">
+        <v>2</v>
       </c>
     </row>
     <row r="73">
@@ -5642,17 +6945,35 @@
       <c r="R73">
         <v>-39.53812623376415</v>
       </c>
+      <c r="S73">
+        <v>-753.4259683304886</v>
+      </c>
       <c r="T73">
-        <v>-753.4259683304886</v>
+        <v>-188.3564920826221</v>
       </c>
       <c r="U73">
-        <v>-188.3564920826221</v>
+        <v>-2009.135915547969</v>
       </c>
       <c r="V73">
-        <v>-2009.135915547969</v>
+        <v>-681.2589220803044</v>
       </c>
       <c r="W73">
-        <v>-681.2589220803044</v>
+        <v>-100.538937531573</v>
+      </c>
+      <c r="X73">
+        <v>-1952.61937759865</v>
+      </c>
+      <c r="Y73">
+        <v>-709.2770434040485</v>
+      </c>
+      <c r="Z73">
+        <v>-128.5570588553172</v>
+      </c>
+      <c r="AA73">
+        <v>-1980.637498922394</v>
+      </c>
+      <c r="AB73">
+        <v>1.9</v>
       </c>
     </row>
     <row r="74">
@@ -5714,17 +7035,35 @@
       <c r="R74">
         <v>-64.03889225641915</v>
       </c>
+      <c r="S74">
+        <v>16.70456314787427</v>
+      </c>
       <c r="T74">
-        <v>16.70456314787427</v>
+        <v>4.176140786968568</v>
       </c>
       <c r="U74">
-        <v>4.176140786968568</v>
+        <v>44.54550172766472</v>
       </c>
       <c r="V74">
-        <v>44.54550172766472</v>
+        <v>271.5840788641179</v>
       </c>
       <c r="W74">
-        <v>271.5840788641179</v>
+        <v>284.4043846880448</v>
+      </c>
+      <c r="X74">
+        <v>274.0762892590757</v>
+      </c>
+      <c r="Y74">
+        <v>253.1091663158553</v>
+      </c>
+      <c r="Z74">
+        <v>265.9294721397822</v>
+      </c>
+      <c r="AA74">
+        <v>255.6013767108132</v>
+      </c>
+      <c r="AB74">
+        <v>6.35593220338983</v>
       </c>
     </row>
     <row r="75">
@@ -5786,17 +7125,35 @@
       <c r="R75">
         <v>-74.28940945752831</v>
       </c>
+      <c r="S75">
+        <v>-420.5163597635979</v>
+      </c>
       <c r="T75">
-        <v>-420.5163597635979</v>
+        <v>-105.1290899408995</v>
       </c>
       <c r="U75">
-        <v>-105.1290899408995</v>
+        <v>-1121.376959369594</v>
       </c>
       <c r="V75">
-        <v>-1121.376959369594</v>
+        <v>-317.7711819779099</v>
       </c>
       <c r="W75">
-        <v>-317.7711819779099</v>
+        <v>27.02231242172678</v>
+      </c>
+      <c r="X75">
+        <v>-1048.038006160844</v>
+      </c>
+      <c r="Y75">
+        <v>-340.4375718152983</v>
+      </c>
+      <c r="Z75">
+        <v>4.355922584338373</v>
+      </c>
+      <c r="AA75">
+        <v>-1070.704395998233</v>
+      </c>
+      <c r="AB75">
+        <v>2</v>
       </c>
     </row>
     <row r="76">
@@ -5858,17 +7215,35 @@
       <c r="R76">
         <v>-70.40174225218152</v>
       </c>
+      <c r="S76">
+        <v>255.4085737801854</v>
+      </c>
       <c r="T76">
-        <v>255.4085737801854</v>
+        <v>63.85214344504634</v>
       </c>
       <c r="U76">
-        <v>63.85214344504634</v>
+        <v>681.0895300804943</v>
       </c>
       <c r="V76">
-        <v>681.0895300804943</v>
+        <v>996.7454575444845</v>
       </c>
       <c r="W76">
-        <v>996.7454575444845</v>
+        <v>833.0563835175005</v>
+      </c>
+      <c r="X76">
+        <v>1394.559057536638</v>
+      </c>
+      <c r="Y76">
+        <v>872.3885314815897</v>
+      </c>
+      <c r="Z76">
+        <v>708.6994574546057</v>
+      </c>
+      <c r="AA76">
+        <v>1270.202131473744</v>
+      </c>
+      <c r="AB76">
+        <v>10.48333333333333</v>
       </c>
     </row>
     <row r="77">
@@ -5930,17 +7305,35 @@
       <c r="R77">
         <v>-75.47952167775412</v>
       </c>
+      <c r="S77">
+        <v>-128.2650949350807</v>
+      </c>
       <c r="T77">
-        <v>-128.2650949350807</v>
+        <v>-32.06627373377018</v>
       </c>
       <c r="U77">
-        <v>-32.06627373377018</v>
+        <v>-342.0402531602153</v>
       </c>
       <c r="V77">
-        <v>-342.0402531602153</v>
+        <v>475.8265392130529</v>
       </c>
       <c r="W77">
-        <v>475.8265392130529</v>
+        <v>601.9026710784744</v>
+      </c>
+      <c r="X77">
+        <v>232.1740703238073</v>
+      </c>
+      <c r="Y77">
+        <v>446.2328801745508</v>
+      </c>
+      <c r="Z77">
+        <v>572.3090120399723</v>
+      </c>
+      <c r="AA77">
+        <v>202.5804112853052</v>
+      </c>
+      <c r="AB77">
+        <v>9.85</v>
       </c>
     </row>
     <row r="78">
@@ -6002,17 +7395,35 @@
       <c r="R78">
         <v>-71.52936454912968</v>
       </c>
+      <c r="S78">
+        <v>-541.6394727238318</v>
+      </c>
       <c r="T78">
-        <v>-541.6394727238318</v>
+        <v>-135.4098681809579</v>
       </c>
       <c r="U78">
-        <v>-135.4098681809579</v>
+        <v>-1444.371927263551</v>
       </c>
       <c r="V78">
-        <v>-1444.371927263551</v>
+        <v>24.43357464627468</v>
       </c>
       <c r="W78">
-        <v>24.43357464627468</v>
+        <v>458.9768859898457</v>
+      </c>
+      <c r="X78">
+        <v>-906.6125866941418</v>
+      </c>
+      <c r="Y78">
+        <v>-10.37012010354783</v>
+      </c>
+      <c r="Z78">
+        <v>424.1731912400232</v>
+      </c>
+      <c r="AA78">
+        <v>-941.4162814439643</v>
+      </c>
+      <c r="AB78">
+        <v>1.9</v>
       </c>
     </row>
     <row r="79">
@@ -6074,17 +7485,35 @@
       <c r="R79">
         <v>-23.96617524080266</v>
       </c>
+      <c r="S79">
+        <v>46.72362019437261</v>
+      </c>
       <c r="T79">
-        <v>46.72362019437261</v>
+        <v>11.68090504859315</v>
       </c>
       <c r="U79">
-        <v>11.68090504859315</v>
+        <v>124.596320518327</v>
       </c>
       <c r="V79">
-        <v>124.596320518327</v>
+        <v>516.7564049834028</v>
       </c>
       <c r="W79">
-        <v>516.7564049834028</v>
+        <v>491.200300870441</v>
+      </c>
+      <c r="X79">
+        <v>585.1424942745394</v>
+      </c>
+      <c r="Y79">
+        <v>485.8209754606559</v>
+      </c>
+      <c r="Z79">
+        <v>460.2648713476941</v>
+      </c>
+      <c r="AA79">
+        <v>554.2070647517926</v>
+      </c>
+      <c r="AB79">
+        <v>2.833333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>